<commit_message>
Added to Do, Updated Pairs
</commit_message>
<xml_diff>
--- a/V2/Pairs_for_Kalshi_and_Polymarket.xlsx
+++ b/V2/Pairs_for_Kalshi_and_Polymarket.xlsx
@@ -1,21 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\davis\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jsher24/Desktop/Traders@SMU/polymarket-copy-trading-bot/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{130D8A54-9B0D-46AE-980D-0D691E454EC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B1FE7F87-70C7-BE42-B038-642D38B19EA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2160" yWindow="2160" windowWidth="19200" windowHeight="11170" xr2:uid="{4F75D300-4D31-744C-B381-2925FE9CB6B9}"/>
+    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16280" xr2:uid="{87DC968E-4842-CC4D-984F-A7EACFB7F109}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <definedNames>
+    <definedName name="tracked_pairs_links" localSheetId="0">Sheet1!$A$1:$I$26</definedName>
+  </definedNames>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -35,65 +38,442 @@
 </workbook>
 </file>
 
+<file path=xl/connections.xml><?xml version="1.0" encoding="utf-8"?>
+<connections xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16">
+  <connection id="1" xr16:uid="{C23EC20A-25F1-C54A-A561-59EE122F401C}" name="tracked_pairs_links" type="6" refreshedVersion="8" background="1" saveData="1">
+    <textPr sourceFile="/Users/jsher24/Desktop/Traders@SMU/polymarket-copy-trading-bot/tracked_pairs_links.csv" tab="0" comma="1">
+      <textFields count="9">
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+      </textFields>
+    </textPr>
+  </connection>
+</connections>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="136">
   <si>
     <t>pair_id</t>
   </si>
   <si>
+    <t>title_clean</t>
+  </si>
+  <si>
+    <t>category_tag</t>
+  </si>
+  <si>
+    <t>similarity_score</t>
+  </si>
+  <si>
     <t>poly_market_id</t>
   </si>
   <si>
+    <t>poly_slug</t>
+  </si>
+  <si>
+    <t>poly_url</t>
+  </si>
+  <si>
     <t>kalshi_market_id</t>
   </si>
   <si>
-    <t>title_clean</t>
-  </si>
-  <si>
-    <t>similarity_score</t>
-  </si>
-  <si>
-    <t>category_tag</t>
-  </si>
-  <si>
-    <t>poly_url</t>
-  </si>
-  <si>
     <t>kalshi_url</t>
   </si>
   <si>
-    <t>poly_slug</t>
+    <t>pair-0001</t>
+  </si>
+  <si>
+    <t>will anthony edwards win the 2025 2026 nba mvp</t>
+  </si>
+  <si>
+    <t>sports</t>
   </si>
   <si>
     <t>will-anthony-edwards-win-the-20252026-nba-mvp</t>
   </si>
   <si>
-    <t>default</t>
-  </si>
-  <si>
-    <t>Will Anthony Edwards win the 2025–2026 NBA MVP?</t>
-  </si>
-  <si>
-    <t>0x33882fdaa147a31a1231293615b6e249ee8cf790fce9d8dc14f312f7b3cc0e30</t>
-  </si>
-  <si>
-    <t>https://polymarket.com/market/will-anthony-edwards-win-the-20252026-nba-mvp</t>
+    <t>https://polymarket.com/event/will-anthony-edwards-win-the-20252026-nba-mvp</t>
+  </si>
+  <si>
+    <t>KXMVECROSSCATEGORY-S2026B8778AB5DFA-8E764236B07</t>
+  </si>
+  <si>
+    <t>https://kalshi.com/markets/KXMVECROSSCATEGORY-S2026B8778AB5DFA-8E764236B07</t>
+  </si>
+  <si>
+    <t>pair-0002</t>
+  </si>
+  <si>
+    <t>will shai gilgeous alexander win the 2025 2026 nba mvp</t>
+  </si>
+  <si>
+    <t>will-shai-gilgeous-alexander-win-the-20252026-nba-mvp</t>
+  </si>
+  <si>
+    <t>https://polymarket.com/event/will-shai-gilgeous-alexander-win-the-20252026-nba-mvp</t>
+  </si>
+  <si>
+    <t>KXMVESPORTSMULTIGAMEEXTENDED-S202686D24CEB3AE-CB0CD9C639F</t>
+  </si>
+  <si>
+    <t>https://kalshi.com/markets/KXMVESPORTSMULTIGAMEEXTENDED-S202686D24CEB3AE-CB0CD9C639F</t>
+  </si>
+  <si>
+    <t>pair-0003</t>
+  </si>
+  <si>
+    <t>will the new orleans pelicans win the 2026 nba finals</t>
+  </si>
+  <si>
+    <t>will-the-new-orleans-pelicans-win-the-2026-nba-finals</t>
+  </si>
+  <si>
+    <t>https://polymarket.com/event/will-the-new-orleans-pelicans-win-the-2026-nba-finals</t>
+  </si>
+  <si>
+    <t>KXMVECROSSCATEGORY-S20269EF9FBC3480-47D2A59B1EE</t>
+  </si>
+  <si>
+    <t>https://kalshi.com/markets/KXMVECROSSCATEGORY-S20269EF9FBC3480-47D2A59B1EE</t>
+  </si>
+  <si>
+    <t>pair-0004</t>
+  </si>
+  <si>
+    <t>will cade cunningham win the 2025 2026 nba mvp</t>
+  </si>
+  <si>
+    <t>will-cade-cunningham-win-the-20252026-nba-mvp</t>
+  </si>
+  <si>
+    <t>https://polymarket.com/event/will-cade-cunningham-win-the-20252026-nba-mvp</t>
+  </si>
+  <si>
+    <t>KXMVECROSSCATEGORY-S2026084A0917FFB-AA1EB963F58</t>
+  </si>
+  <si>
+    <t>https://kalshi.com/markets/KXMVECROSSCATEGORY-S2026084A0917FFB-AA1EB963F58</t>
+  </si>
+  <si>
+    <t>pair-0005</t>
+  </si>
+  <si>
+    <t>will jaylen brown win the 2025 2026 nba mvp</t>
+  </si>
+  <si>
+    <t>will-jaylen-brown-win-the-20252026-nba-mvp</t>
+  </si>
+  <si>
+    <t>https://polymarket.com/event/will-jaylen-brown-win-the-20252026-nba-mvp</t>
+  </si>
+  <si>
+    <t>KXMVECROSSCATEGORY-S2026886F9862E1F-C6FFDD876E0</t>
+  </si>
+  <si>
+    <t>https://kalshi.com/markets/KXMVECROSSCATEGORY-S2026886F9862E1F-C6FFDD876E0</t>
+  </si>
+  <si>
+    <t>pair-0006</t>
+  </si>
+  <si>
+    <t>will the los angeles kings win the 2026 nhl stanley cup</t>
+  </si>
+  <si>
+    <t>will-the-los-angeles-kings-win-the-2026-nhl-stanley-cup</t>
+  </si>
+  <si>
+    <t>https://polymarket.com/event/will-the-los-angeles-kings-win-the-2026-nhl-stanley-cup</t>
+  </si>
+  <si>
+    <t>KXMVECROSSCATEGORY-S20263A9D95419E6-C33AA0320A8</t>
+  </si>
+  <si>
+    <t>https://kalshi.com/markets/KXMVECROSSCATEGORY-S20263A9D95419E6-C33AA0320A8</t>
+  </si>
+  <si>
+    <t>pair-0007</t>
+  </si>
+  <si>
+    <t>will lebron james win the 2028 democratic presidential nomination</t>
+  </si>
+  <si>
+    <t>politics</t>
+  </si>
+  <si>
+    <t>will-lebron-james-win-the-2028-democratic-presidential-nomination</t>
+  </si>
+  <si>
+    <t>https://polymarket.com/event/will-lebron-james-win-the-2028-democratic-presidential-nomination</t>
+  </si>
+  <si>
+    <t>KXMVECROSSCATEGORY-S20264F2FAE36450-8279BDF825B</t>
+  </si>
+  <si>
+    <t>https://kalshi.com/markets/KXMVECROSSCATEGORY-S20264F2FAE36450-8279BDF825B</t>
+  </si>
+  <si>
+    <t>pair-0008</t>
+  </si>
+  <si>
+    <t>will real madrid win the 2025 26 champions league</t>
+  </si>
+  <si>
+    <t>other</t>
+  </si>
+  <si>
+    <t>will-real-madrid-win-the-202526-champions-league</t>
+  </si>
+  <si>
+    <t>https://polymarket.com/event/will-real-madrid-win-the-202526-champions-league</t>
+  </si>
+  <si>
+    <t>KXMVECROSSCATEGORY-S2026CD65ABB47E5-A857D99647F</t>
+  </si>
+  <si>
+    <t>https://kalshi.com/markets/KXMVECROSSCATEGORY-S2026CD65ABB47E5-A857D99647F</t>
   </si>
   <si>
     <t>pair-0009</t>
   </si>
   <si>
-    <t>KXNBAMVP-26-AEDW</t>
-  </si>
-  <si>
-    <t>https://kalshi.com/markets/KXNBAMVP-26-AEDW</t>
+    <t>will the oklahoma city thunder win the 2026 nba finals</t>
+  </si>
+  <si>
+    <t>will-the-oklahoma-city-thunder-win-the-2026-nba-finals</t>
+  </si>
+  <si>
+    <t>https://polymarket.com/event/will-the-oklahoma-city-thunder-win-the-2026-nba-finals</t>
+  </si>
+  <si>
+    <t>KXMVECROSSCATEGORY-S202679CF7D60E0F-C290E82693C</t>
+  </si>
+  <si>
+    <t>https://kalshi.com/markets/KXMVECROSSCATEGORY-S202679CF7D60E0F-C290E82693C</t>
+  </si>
+  <si>
+    <t>pair-0010</t>
+  </si>
+  <si>
+    <t>will tyrese maxey win the 2025 2026 nba mvp</t>
+  </si>
+  <si>
+    <t>will-tyrese-maxey-win-the-20252026-nba-mvp</t>
+  </si>
+  <si>
+    <t>https://polymarket.com/event/will-tyrese-maxey-win-the-20252026-nba-mvp</t>
+  </si>
+  <si>
+    <t>KXMVECROSSCATEGORY-S2026D37CBF334D1-B7797C46DB2</t>
+  </si>
+  <si>
+    <t>https://kalshi.com/markets/KXMVECROSSCATEGORY-S2026D37CBF334D1-B7797C46DB2</t>
+  </si>
+  <si>
+    <t>pair-0011</t>
+  </si>
+  <si>
+    <t>will bayern munich win the 2025 26 champions league</t>
+  </si>
+  <si>
+    <t>will-bayern-munich-win-the-202526-champions-league</t>
+  </si>
+  <si>
+    <t>https://polymarket.com/event/will-bayern-munich-win-the-202526-champions-league</t>
+  </si>
+  <si>
+    <t>KXMVECROSSCATEGORY-S2026D04FC0A1D8D-F19E1E0A84A</t>
+  </si>
+  <si>
+    <t>https://kalshi.com/markets/KXMVECROSSCATEGORY-S2026D04FC0A1D8D-F19E1E0A84A</t>
+  </si>
+  <si>
+    <t>pair-0012</t>
+  </si>
+  <si>
+    <t>will the new york rangers win the 2026 nhl stanley cup</t>
+  </si>
+  <si>
+    <t>will-the-new-york-rangers-win-the-2026-nhl-stanley-cup</t>
+  </si>
+  <si>
+    <t>https://polymarket.com/event/will-the-new-york-rangers-win-the-2026-nhl-stanley-cup</t>
+  </si>
+  <si>
+    <t>KXMVECROSSCATEGORY-S2026286BEFF7D0B-CF636424568</t>
+  </si>
+  <si>
+    <t>https://kalshi.com/markets/KXMVECROSSCATEGORY-S2026286BEFF7D0B-CF636424568</t>
+  </si>
+  <si>
+    <t>pair-0013</t>
+  </si>
+  <si>
+    <t>will dortmund win the 2025 26 bundesliga</t>
+  </si>
+  <si>
+    <t>will-dortmund-win-the-202526-bundesliga</t>
+  </si>
+  <si>
+    <t>https://polymarket.com/event/will-dortmund-win-the-202526-bundesliga</t>
+  </si>
+  <si>
+    <t>KXMVECROSSCATEGORY-S202692EFD37F4E2-7935C052F97</t>
+  </si>
+  <si>
+    <t>https://kalshi.com/markets/KXMVECROSSCATEGORY-S202692EFD37F4E2-7935C052F97</t>
+  </si>
+  <si>
+    <t>pair-0014</t>
+  </si>
+  <si>
+    <t>new rihanna album before gta vi</t>
+  </si>
+  <si>
+    <t>new-rhianna-album-before-gta-vi-926</t>
+  </si>
+  <si>
+    <t>https://polymarket.com/event/new-rhianna-album-before-gta-vi-926</t>
+  </si>
+  <si>
+    <t>KXMVECROSSCATEGORY-S20264C795D7A4D0-13DB55E5D1C</t>
+  </si>
+  <si>
+    <t>https://kalshi.com/markets/KXMVECROSSCATEGORY-S20264C795D7A4D0-13DB55E5D1C</t>
+  </si>
+  <si>
+    <t>pair-0015</t>
+  </si>
+  <si>
+    <t>KXMVECROSSCATEGORY-S20266FEA88A399C-95EF8FC89FA</t>
+  </si>
+  <si>
+    <t>https://kalshi.com/markets/KXMVECROSSCATEGORY-S20266FEA88A399C-95EF8FC89FA</t>
+  </si>
+  <si>
+    <t>pair-0016</t>
+  </si>
+  <si>
+    <t>KXMVECROSSCATEGORY-S20269129EBB8407-0DD75E131F0</t>
+  </si>
+  <si>
+    <t>https://kalshi.com/markets/KXMVECROSSCATEGORY-S20269129EBB8407-0DD75E131F0</t>
+  </si>
+  <si>
+    <t>pair-0017</t>
+  </si>
+  <si>
+    <t>will the carolina hurricanes win the 2026 nhl stanley cup</t>
+  </si>
+  <si>
+    <t>will-the-carolina-hurricanes-win-the-2026-nhl-stanley-cup</t>
+  </si>
+  <si>
+    <t>https://polymarket.com/event/will-the-carolina-hurricanes-win-the-2026-nhl-stanley-cup</t>
+  </si>
+  <si>
+    <t>KXMVECROSSCATEGORY-S20262C88EEABD53-B63A1EF7391</t>
+  </si>
+  <si>
+    <t>https://kalshi.com/markets/KXMVECROSSCATEGORY-S20262C88EEABD53-B63A1EF7391</t>
+  </si>
+  <si>
+    <t>pair-0018</t>
+  </si>
+  <si>
+    <t>KXMVECROSSCATEGORY-S202644C863E6EF2-0A7CDCE94C1</t>
+  </si>
+  <si>
+    <t>https://kalshi.com/markets/KXMVECROSSCATEGORY-S202644C863E6EF2-0A7CDCE94C1</t>
+  </si>
+  <si>
+    <t>pair-0019</t>
+  </si>
+  <si>
+    <t>KXMVECROSSCATEGORY-S2026C7A2D2069BB-9A6B57659B1</t>
+  </si>
+  <si>
+    <t>https://kalshi.com/markets/KXMVECROSSCATEGORY-S2026C7A2D2069BB-9A6B57659B1</t>
+  </si>
+  <si>
+    <t>pair-0020</t>
+  </si>
+  <si>
+    <t>KXMVECROSSCATEGORY-S20267CD770A6736-1B2210915AB</t>
+  </si>
+  <si>
+    <t>https://kalshi.com/markets/KXMVECROSSCATEGORY-S20267CD770A6736-1B2210915AB</t>
+  </si>
+  <si>
+    <t>pair-0021</t>
+  </si>
+  <si>
+    <t>KXMVECROSSCATEGORY-S20265773B80332E-2A7CB463315</t>
+  </si>
+  <si>
+    <t>https://kalshi.com/markets/KXMVECROSSCATEGORY-S20265773B80332E-2A7CB463315</t>
+  </si>
+  <si>
+    <t>pair-0022</t>
+  </si>
+  <si>
+    <t>KXMVECROSSCATEGORY-S2026E699A91E46C-FA16BD2B650</t>
+  </si>
+  <si>
+    <t>https://kalshi.com/markets/KXMVECROSSCATEGORY-S2026E699A91E46C-FA16BD2B650</t>
+  </si>
+  <si>
+    <t>pair-0023</t>
+  </si>
+  <si>
+    <t>will the florida panthers win the 2026 nhl stanley cup</t>
+  </si>
+  <si>
+    <t>will-the-florida-panthers-win-the-2026-nhl-stanley-cup</t>
+  </si>
+  <si>
+    <t>https://polymarket.com/event/will-the-florida-panthers-win-the-2026-nhl-stanley-cup</t>
+  </si>
+  <si>
+    <t>KXMVECROSSCATEGORY-S202678CC5B2637C-BECFF231FBC</t>
+  </si>
+  <si>
+    <t>https://kalshi.com/markets/KXMVECROSSCATEGORY-S202678CC5B2637C-BECFF231FBC</t>
+  </si>
+  <si>
+    <t>pair-0024</t>
+  </si>
+  <si>
+    <t>KXMVECROSSCATEGORY-S2026775CB00200D-10DF48D3E3F</t>
+  </si>
+  <si>
+    <t>https://kalshi.com/markets/KXMVECROSSCATEGORY-S2026775CB00200D-10DF48D3E3F</t>
+  </si>
+  <si>
+    <t>pair-0025</t>
+  </si>
+  <si>
+    <t>KXMVECROSSCATEGORY-S2026EAC63F803B6-582E9DB1C12</t>
+  </si>
+  <si>
+    <t>https://kalshi.com/markets/KXMVECROSSCATEGORY-S2026EAC63F803B6-582E9DB1C12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Time to expiration (2 months out) </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -101,21 +481,19 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <u/>
-      <sz val="12"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -127,16 +505,14 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -152,10 +528,14 @@
 </styleSheet>
 </file>
 
+<file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="tracked_pairs_links" connectionId="1" xr16:uid="{51C24B16-09C0-204E-B6A8-A5ABF8C181F7}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -193,7 +573,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -299,7 +679,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -441,84 +821,784 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FECAC60-48D7-43F9-806E-3C5F68959A94}">
-  <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B3B2B3B-E1EC-0F45-9EEF-1EAC6924D9DF}">
+  <dimension ref="A1:K26"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.58203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="44.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.4140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.75" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="65.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="42.83203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="70.4140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.75" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="42.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="57.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="59" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="80.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="63.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="80.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="24.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
         <v>5</v>
-      </c>
-      <c r="D1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F1" t="s">
-        <v>8</v>
       </c>
       <c r="G1" t="s">
         <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+      <c r="K1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
         <v>11</v>
       </c>
-      <c r="C2" t="s">
-        <v>10</v>
-      </c>
       <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2" t="s">
+        <v>0.18179999999999999</v>
+      </c>
+      <c r="E2">
+        <v>564165</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
       </c>
       <c r="G2" t="s">
         <v>13</v>
       </c>
       <c r="H2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="1" t="s">
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>0.17649999999999999</v>
+      </c>
+      <c r="E3">
+        <v>564162</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4">
+        <v>0.16669999999999999</v>
+      </c>
+      <c r="E4">
+        <v>553875</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" t="s">
+        <v>26</v>
+      </c>
+      <c r="I4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5">
+        <v>0.16669999999999999</v>
+      </c>
+      <c r="E5">
+        <v>564168</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="G5" t="s">
+        <v>31</v>
+      </c>
+      <c r="H5" t="s">
+        <v>32</v>
+      </c>
+      <c r="I5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6">
+        <v>0.16669999999999999</v>
+      </c>
+      <c r="E6">
+        <v>564175</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G6" t="s">
+        <v>37</v>
+      </c>
+      <c r="H6" t="s">
+        <v>38</v>
+      </c>
+      <c r="I6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7">
+        <v>0.15379999999999999</v>
+      </c>
+      <c r="E7">
+        <v>553831</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="G7" t="s">
+        <v>43</v>
+      </c>
+      <c r="H7" t="s">
+        <v>44</v>
+      </c>
+      <c r="I7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D8">
+        <v>0.15379999999999999</v>
+      </c>
+      <c r="E8">
+        <v>559681</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G8" t="s">
+        <v>50</v>
+      </c>
+      <c r="H8" t="s">
+        <v>51</v>
+      </c>
+      <c r="I8" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" t="s">
+        <v>54</v>
+      </c>
+      <c r="C9" t="s">
+        <v>55</v>
+      </c>
+      <c r="D9">
+        <v>0.15379999999999999</v>
+      </c>
+      <c r="E9">
+        <v>566139</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="G9" t="s">
+        <v>57</v>
+      </c>
+      <c r="H9" t="s">
+        <v>58</v>
+      </c>
+      <c r="I9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>60</v>
+      </c>
+      <c r="B10" t="s">
+        <v>61</v>
+      </c>
+      <c r="C10" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10">
+        <v>0.1429</v>
+      </c>
+      <c r="E10">
+        <v>553856</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="G10" t="s">
+        <v>63</v>
+      </c>
+      <c r="H10" t="s">
+        <v>64</v>
+      </c>
+      <c r="I10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>66</v>
+      </c>
+      <c r="B11" t="s">
+        <v>67</v>
+      </c>
+      <c r="C11" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11">
+        <v>0.1333</v>
+      </c>
+      <c r="E11">
+        <v>564183</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="G11" t="s">
+        <v>69</v>
+      </c>
+      <c r="H11" t="s">
+        <v>70</v>
+      </c>
+      <c r="I11" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>72</v>
+      </c>
+      <c r="B12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C12" t="s">
+        <v>55</v>
+      </c>
+      <c r="D12">
+        <v>0.1333</v>
+      </c>
+      <c r="E12">
+        <v>566142</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="G12" t="s">
+        <v>75</v>
+      </c>
+      <c r="H12" t="s">
+        <v>76</v>
+      </c>
+      <c r="I12" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>78</v>
+      </c>
+      <c r="B13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C13" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13">
+        <v>0.125</v>
+      </c>
+      <c r="E13">
+        <v>553836</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="G13" t="s">
+        <v>81</v>
+      </c>
+      <c r="H13" t="s">
+        <v>82</v>
+      </c>
+      <c r="I13" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>84</v>
+      </c>
+      <c r="B14" t="s">
+        <v>85</v>
+      </c>
+      <c r="C14" t="s">
+        <v>55</v>
+      </c>
+      <c r="D14">
+        <v>0.125</v>
+      </c>
+      <c r="E14">
+        <v>566538</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="G14" t="s">
+        <v>87</v>
+      </c>
+      <c r="H14" t="s">
+        <v>88</v>
+      </c>
+      <c r="I14" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>90</v>
+      </c>
+      <c r="B15" t="s">
+        <v>91</v>
+      </c>
+      <c r="C15" t="s">
+        <v>55</v>
+      </c>
+      <c r="D15">
+        <v>7.1400000000000005E-2</v>
+      </c>
+      <c r="E15">
+        <v>540817</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G15" t="s">
+        <v>93</v>
+      </c>
+      <c r="H15" t="s">
+        <v>94</v>
+      </c>
+      <c r="I15" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>96</v>
+      </c>
+      <c r="B16" t="s">
+        <v>91</v>
+      </c>
+      <c r="C16" t="s">
+        <v>55</v>
+      </c>
+      <c r="D16">
+        <v>7.1400000000000005E-2</v>
+      </c>
+      <c r="E16">
+        <v>540817</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G16" t="s">
+        <v>93</v>
+      </c>
+      <c r="H16" t="s">
+        <v>97</v>
+      </c>
+      <c r="I16" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>99</v>
+      </c>
+      <c r="B17" t="s">
+        <v>91</v>
+      </c>
+      <c r="C17" t="s">
+        <v>55</v>
+      </c>
+      <c r="D17">
+        <v>6.6699999999999995E-2</v>
+      </c>
+      <c r="E17">
+        <v>540817</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G17" t="s">
+        <v>93</v>
+      </c>
+      <c r="H17" t="s">
+        <v>100</v>
+      </c>
+      <c r="I17" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>102</v>
+      </c>
+      <c r="B18" t="s">
+        <v>103</v>
+      </c>
+      <c r="C18" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18">
+        <v>6.6699999999999995E-2</v>
+      </c>
+      <c r="E18">
+        <v>553824</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G18" t="s">
+        <v>105</v>
+      </c>
+      <c r="H18" t="s">
+        <v>106</v>
+      </c>
+      <c r="I18" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>108</v>
+      </c>
+      <c r="B19" t="s">
+        <v>91</v>
+      </c>
+      <c r="C19" t="s">
+        <v>55</v>
+      </c>
+      <c r="D19">
+        <v>6.25E-2</v>
+      </c>
+      <c r="E19">
+        <v>540817</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G19" t="s">
+        <v>93</v>
+      </c>
+      <c r="H19" t="s">
+        <v>109</v>
+      </c>
+      <c r="I19" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>111</v>
+      </c>
+      <c r="B20" t="s">
+        <v>103</v>
+      </c>
+      <c r="C20" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20">
+        <v>5.8799999999999998E-2</v>
+      </c>
+      <c r="E20">
+        <v>553824</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G20" t="s">
+        <v>105</v>
+      </c>
+      <c r="H20" t="s">
+        <v>112</v>
+      </c>
+      <c r="I20" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>114</v>
+      </c>
+      <c r="B21" t="s">
+        <v>103</v>
+      </c>
+      <c r="C21" t="s">
+        <v>11</v>
+      </c>
+      <c r="D21">
+        <v>5.8799999999999998E-2</v>
+      </c>
+      <c r="E21">
+        <v>553824</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G21" t="s">
+        <v>105</v>
+      </c>
+      <c r="H21" t="s">
+        <v>115</v>
+      </c>
+      <c r="I21" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>117</v>
+      </c>
+      <c r="B22" t="s">
+        <v>91</v>
+      </c>
+      <c r="C22" t="s">
+        <v>55</v>
+      </c>
+      <c r="D22">
+        <v>5.5599999999999997E-2</v>
+      </c>
+      <c r="E22">
+        <v>540817</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G22" t="s">
+        <v>93</v>
+      </c>
+      <c r="H22" t="s">
+        <v>118</v>
+      </c>
+      <c r="I22" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>120</v>
+      </c>
+      <c r="B23" t="s">
+        <v>91</v>
+      </c>
+      <c r="C23" t="s">
+        <v>55</v>
+      </c>
+      <c r="D23">
+        <v>5.5599999999999997E-2</v>
+      </c>
+      <c r="E23">
+        <v>540817</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G23" t="s">
+        <v>93</v>
+      </c>
+      <c r="H23" t="s">
+        <v>121</v>
+      </c>
+      <c r="I23" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>123</v>
+      </c>
+      <c r="B24" t="s">
+        <v>124</v>
+      </c>
+      <c r="C24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24">
+        <v>5.5599999999999997E-2</v>
+      </c>
+      <c r="E24">
+        <v>553825</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="G24" t="s">
+        <v>126</v>
+      </c>
+      <c r="H24" t="s">
+        <v>127</v>
+      </c>
+      <c r="I24" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>129</v>
+      </c>
+      <c r="B25" t="s">
+        <v>91</v>
+      </c>
+      <c r="C25" t="s">
+        <v>55</v>
+      </c>
+      <c r="D25">
+        <v>5.2600000000000001E-2</v>
+      </c>
+      <c r="E25">
+        <v>540817</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G25" t="s">
+        <v>93</v>
+      </c>
+      <c r="H25" t="s">
+        <v>130</v>
+      </c>
+      <c r="I25" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>132</v>
+      </c>
+      <c r="B26" t="s">
+        <v>103</v>
+      </c>
+      <c r="C26" t="s">
+        <v>11</v>
+      </c>
+      <c r="D26">
+        <v>5.2600000000000001E-2</v>
+      </c>
+      <c r="E26">
+        <v>553824</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G26" t="s">
+        <v>105</v>
+      </c>
+      <c r="H26" t="s">
+        <v>133</v>
+      </c>
+      <c r="I26" t="s">
+        <v>134</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
NC State vs. Texas
</commit_message>
<xml_diff>
--- a/V2/Pairs_for_Kalshi_and_Polymarket.xlsx
+++ b/V2/Pairs_for_Kalshi_and_Polymarket.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1161"/>
+  <dimension ref="A1:K1162"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
     <col width="9" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -51838,6 +51838,53 @@
         </is>
       </c>
     </row>
+    <row r="1162">
+      <c r="A1162" t="inlineStr">
+        <is>
+          <t>pair-0172</t>
+        </is>
+      </c>
+      <c r="B1162" t="inlineStr">
+        <is>
+          <t>North Carolina State Wolfpack vs. Texas Longhorns</t>
+        </is>
+      </c>
+      <c r="C1162" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="D1162" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="E1162" t="inlineStr">
+        <is>
+          <t>0x68cbb3bd267f30f766bc22ae7dd3ea0263c3abe3dc769eb63f98a12cd3b7ebfb</t>
+        </is>
+      </c>
+      <c r="F1162" t="inlineStr">
+        <is>
+          <t>cbb-ncst-tx-2026-03-17</t>
+        </is>
+      </c>
+      <c r="G1162" t="inlineStr">
+        <is>
+          <t>https://polymarket.com/market/cbb-ncst-tx-2026-03-17</t>
+        </is>
+      </c>
+      <c r="H1162" t="inlineStr">
+        <is>
+          <t>KXNCAAMBGAME-26MAR17TEXNCST-TEX</t>
+        </is>
+      </c>
+      <c r="I1162" t="inlineStr">
+        <is>
+          <t>https://kalshi.com/markets/KXNCAAMBGAME-26MAR17TEXNCST-TEX</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId1"/>

</xml_diff>

<commit_message>
Fed Interest Rates (April)
</commit_message>
<xml_diff>
--- a/V2/Pairs_for_Kalshi_and_Polymarket.xlsx
+++ b/V2/Pairs_for_Kalshi_and_Polymarket.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1207"/>
+  <dimension ref="A1:K1208"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
     <col width="9" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -54000,6 +54000,53 @@
         </is>
       </c>
     </row>
+    <row r="1208">
+      <c r="A1208" t="inlineStr">
+        <is>
+          <t>pair-0223</t>
+        </is>
+      </c>
+      <c r="B1208" t="inlineStr">
+        <is>
+          <t>Will there be no change in Fed interest rates after the April 2026 meeting?</t>
+        </is>
+      </c>
+      <c r="C1208" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="D1208" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="E1208" t="inlineStr">
+        <is>
+          <t>0x36e8ca24d2a13435f519f15580d42b45cdbe3bc425fb39a7c2733260357af0fa</t>
+        </is>
+      </c>
+      <c r="F1208" t="inlineStr">
+        <is>
+          <t>will-there-be-no-change-in-fed-interest-rates-after-the-april-2026-meeting</t>
+        </is>
+      </c>
+      <c r="G1208" t="inlineStr">
+        <is>
+          <t>https://polymarket.com/market/will-there-be-no-change-in-fed-interest-rates-after-the-april-2026-meeting</t>
+        </is>
+      </c>
+      <c r="H1208" t="inlineStr">
+        <is>
+          <t>KXFEDDECISION-26APR-H0</t>
+        </is>
+      </c>
+      <c r="I1208" t="inlineStr">
+        <is>
+          <t>https://kalshi.com/markets/KXFEDDECISION-26APR-H0</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId1"/>

</xml_diff>